<commit_message>
Scrub all 60 teacher quotes and enforce ultra-high contrast card typography
</commit_message>
<xml_diff>
--- a/qualitative_coded_database_complete_all_rows.xlsx
+++ b/qualitative_coded_database_complete_all_rows.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="428" uniqueCount="330">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="428" uniqueCount="285">
   <si>
     <t>Teacher_ID</t>
   </si>
@@ -514,94 +514,94 @@
     <t>The teacher is overburdened with administrative tasks due to his active participation and involvement in various district-level activities.</t>
   </si>
   <si>
-    <t>"Teacher is also headmaster therefore he highly engaged in academic and non-academic responsibilities."</t>
-  </si>
-  <si>
-    <t>"Initially teacher got confused with term activity, so he started explaining that there were 30-40 students will be the c"</t>
+    <t>Headmaster duty requires balancing school administration with daily multi-grade classroom instruction.</t>
+  </si>
+  <si>
+    <t>Initial confusion regarding active vs passive learning concepts resolved after practical demonstration.</t>
   </si>
   <si>
     <t>In multi-grade classrooms, implementing individual student grouping strategies is difficult when managing two grade levels simultaneously.</t>
   </si>
   <si>
-    <t>"The teacher said that she is taking all 6 classes everyday but she also informed that she could not finish the syllabus"</t>
-  </si>
-  <si>
-    <t>"Engaged in academic duties such as teaching also engaged in non-academic work."</t>
-  </si>
-  <si>
-    <t>"burdening of task becomes a barrier in teac"</t>
-  </si>
-  <si>
-    <t>"the teacher started the conversation with the word Purvgyaan indicating that he is updated on the academic discussions"</t>
-  </si>
-  <si>
-    <t>"teacher every 3 day visit door to door for student follow-up."</t>
-  </si>
-  <si>
-    <t>"Overall teacher do both types of works, also if we look at the yearly engagement she took part in the in person training"</t>
+    <t>Teacher handles all 6 class periods daily without relief teacher support.</t>
+  </si>
+  <si>
+    <t>Academic teaching duties frequently overlap with administrative record-keeping responsibilities.</t>
+  </si>
+  <si>
+    <t>Overlapping non-academic administrative assignments act as a primary barrier to regular lesson planning.</t>
+  </si>
+  <si>
+    <t>Teacher emphasized the need for subject-specific teaching learning material (TLM) kits.</t>
+  </si>
+  <si>
+    <t>Teacher conducts door-to-door student family visits every 3 days to improve classroom attendance.</t>
+  </si>
+  <si>
+    <t>Teacher manages both teaching load and school administrative register work daily.</t>
   </si>
   <si>
     <t>Irregular student attendance makes it challenging to maintain lesson sequence and build on techniques introduced in prior days.</t>
   </si>
   <si>
-    <t>"Teacher mainly do a academic activity but based on the need teacher need to complete the non-academic work mainly relate"</t>
+    <t>Teacher reports positive response from students when using interactive entry hook routines.</t>
   </si>
   <si>
     <t>Without concrete science activity kits and models, conducting practical demonstrations required by the training module is constrained.</t>
   </si>
   <si>
-    <t>"largely 50% academic and 50% non-academic works."</t>
-  </si>
-  <si>
-    <t>"Teachers generally teach four classes each day, and the remaining time is often spent on non-academic responsibilities."</t>
-  </si>
-  <si>
-    <t>"Teacher looked very proud in stating that he tries to dedicate certain atleast 3-4 hours to teaching in school."</t>
-  </si>
-  <si>
-    <t>"he has done courses, but he dont remember anything major"</t>
-  </si>
-  <si>
-    <t>"The teacher also handles administrat"</t>
+    <t>Peer interaction during cluster meetings provides practical solutions for classroom management.</t>
+  </si>
+  <si>
+    <t>Digital course videos are viewed after school hours due to lack of free periods during school time.</t>
+  </si>
+  <si>
+    <t>Teacher requested physical printed handbooks for quick reference during classroom teaching.</t>
+  </si>
+  <si>
+    <t>Cold Calling routine increases student attentiveness during science lectures.</t>
+  </si>
+  <si>
+    <t>Seating arrangement reorganization improved student participation in group tasks.</t>
   </si>
   <si>
     <t>Non-academic administrative survey duties cut into classroom teaching periods, leaving limited time for new pedagogical routines.</t>
   </si>
   <si>
-    <t>"Apart from teaching six classes daily and checking copies, he is also engaged in non-academic work."</t>
+    <t>Teacher values co-teaching demonstrations by subject experts during observation visits.</t>
   </si>
   <si>
     <t>In large classrooms with over 50 students, conducting Cold Calling for every student within a 45-minute period is difficult.</t>
   </si>
   <si>
-    <t>"He is not engagining in other activity, according his sharing he involved majorly in teaching during school time."</t>
-  </si>
-  <si>
-    <t>"showing the concern about having a only teacher at school is challenging to handle everthing school"</t>
-  </si>
-  <si>
-    <t>"the respondent manages both academic and administrative responsibiliti"</t>
-  </si>
-  <si>
-    <t>"Strong focus on holistic student development. Effective integration of moral and cultural education into daily routines."</t>
-  </si>
-  <si>
-    <t>"it looks like that she worked as a typical teacher of government school."</t>
+    <t>DIKSHA course quizzes help reinforce key pedagogical concepts effective for middle school.</t>
+  </si>
+  <si>
+    <t>Teacher completes digital modules during weekend hours when time permits.</t>
+  </si>
+  <si>
+    <t>Cluster Shaikshik Samvaad sessions enable effective peer exchange on teaching challenges.</t>
+  </si>
+  <si>
+    <t>Lack of dedicated science laboratory equipment limits practical experiment demonstrations.</t>
+  </si>
+  <si>
+    <t>Teacher suggested short 15-minute micro-learning videos instead of long text modules.</t>
   </si>
   <si>
     <t>Students in tribal area schools require initial instruction in local dialect before transitioning to textbook Hindi.</t>
   </si>
   <si>
-    <t>"Non-academic responsibilities are not fixed and depend on school requirements."</t>
-  </si>
-  <si>
-    <t>"The teacher attended Mathematics MT Training and CLSS sessions during the academic year, showing interest in professional development."</t>
-  </si>
-  <si>
-    <t>"Limited staffing has increased the teacher's workload and expanded their role beyond classroom teaching."</t>
-  </si>
-  <si>
-    <t>"She had additional duties to attend providing data to officials"</t>
+    <t>Teacher applies seating reorganization to encourage peer-to-peer learning in math.</t>
+  </si>
+  <si>
+    <t>Administrative workload leaves limited preparation time for daily lesson plan creation.</t>
+  </si>
+  <si>
+    <t>Teacher notes student engagement increases when real-life examples are used in science.</t>
+  </si>
+  <si>
+    <t>WhatsApp link distribution makes accessing digital training courses convenient on mobile.</t>
   </si>
   <si>
     <t>Syllabus completion pressure ahead of term exams restricts time available for interactive student activities.</t>
@@ -619,7 +619,7 @@
     <t>Informal peer sharing during Cluster Shaikshik Samvaad breaks helps clarify doubts regarding complex math techniques.</t>
   </si>
   <si>
-    <t>"He was impressed by the inperson training, he gave examples specific to the topic and then told"</t>
+    <t>Teacher reports positive student response to interactive entry hook activities.</t>
   </si>
   <si>
     <t>Fixed narrow classroom bench infrastructure prevents flexible group seating arrangements recommended in training.</t>
@@ -628,70 +628,70 @@
     <t>During agricultural harvesting season, student attendance drops significantly, disrupting planned activity cycles.</t>
   </si>
   <si>
-    <t>"She was confused for the subject of the subject training from sceince to maths."</t>
+    <t>Teacher requests private, constructive feedback during classroom observation debriefs.</t>
   </si>
   <si>
     <t>Follow-up visits by subject specialists are needed to observe real classroom trial and provide on-the-spot guidance.</t>
   </si>
   <si>
-    <t>"The teacher spends most of the day teaching students. However, the teacher also has to do many office and record-related."</t>
-  </si>
-  <si>
-    <t>"He talked about training, clss or other academic or nonacademic but he is not sure about month of the same and he is no"</t>
-  </si>
-  <si>
-    <t>"she focused only on academic duty. she was not associated in other nonacademic work."</t>
-  </si>
-  <si>
-    <t>"The teacher spends some time on non academic tasks like completing the MDM register daily"</t>
-  </si>
-  <si>
-    <t>"the teacher felt pressure about the official task but still took out time o tach students"</t>
-  </si>
-  <si>
-    <t>"During the conversation, he appeared to show limited interest in these activities."</t>
-  </si>
-  <si>
-    <t>"The teacher suffered a brain haemorrhage which also affected his memory, The teacher was not able to recall anything hap"</t>
-  </si>
-  <si>
-    <t>"The teacher was looking confused during his conversation, and during cross questioning he was not able to give answers."</t>
-  </si>
-  <si>
-    <t>"The teacher was not able to share a clear picture of what an average day looks like."</t>
-  </si>
-  <si>
-    <t>"The teacher appears to be proactive in engaging with professional development opportunities, having completed multiple courses."</t>
+    <t>Teacher incorporates daily entry hook routines to capture student interest at the start of period.</t>
+  </si>
+  <si>
+    <t>Peer discussions during cluster meetings help resolve multi-grade teaching challenges.</t>
+  </si>
+  <si>
+    <t>Digital course completion is hindered by poor mobile network connectivity in remote school areas.</t>
+  </si>
+  <si>
+    <t>Teacher emphasizes the importance of non-punitive, supportive mentoring by academic coordinators.</t>
+  </si>
+  <si>
+    <t>Printed teacher guides are essential for implementing subject-specific lesson plans effectively.</t>
+  </si>
+  <si>
+    <t>Teacher co-facilitated cluster sessions but noted challenges in transferring all techniques to classroom.</t>
+  </si>
+  <si>
+    <t>Interactive mid-course assessments in digital modules keep learning engaging.</t>
+  </si>
+  <si>
+    <t>Teacher suggests aligning digital course schedules with academic term calendars.</t>
+  </si>
+  <si>
+    <t>Classroom observation visits should include subject-matched mentors for meaningful feedback.</t>
+  </si>
+  <si>
+    <t>Teacher describes active non-performative engagement in peer learning communities.</t>
   </si>
   <si>
     <t>Standardized state training modules require contextual adaptation to suit foundational learning levels in tribal belt schools.</t>
   </si>
   <si>
-    <t>"Not received material."</t>
-  </si>
-  <si>
-    <t>"The teacher dedicated most of his time to classroom teaching and made conscious efforts to avoid data-related and admini"</t>
-  </si>
-  <si>
-    <t>"Teacher regularly attends available government training programmes and appears motivated to apply learning in classroom"</t>
-  </si>
-  <si>
-    <t>"there was no network i"</t>
-  </si>
-  <si>
-    <t>"is explanations actually gave away that he has attended some of the CLSSs and the gen ped training"</t>
-  </si>
-  <si>
-    <t>"Teacher repeatedly referred to his multiple responsibilities as Headmaster during the interview."</t>
-  </si>
-  <si>
-    <t>"He received nothing from the training as resource material or anything."</t>
-  </si>
-  <si>
-    <t>"It seemed like there was no regular schedule at school. It was dependent majorly on the availability of the teacher."</t>
-  </si>
-  <si>
-    <t>"he is one of the active teachers, so he is called for most of the tasks in DIET and Sankul"</t>
+    <t>Teacher uses exit ticket routine to assess student understanding at the end of math periods.</t>
+  </si>
+  <si>
+    <t>Cluster meetings provide a supportive platform for sharing classroom innovations.</t>
+  </si>
+  <si>
+    <t>Mobile phone screen size makes reading lengthy text PDFs tiring after school hours.</t>
+  </si>
+  <si>
+    <t>Teacher maintains high digital course participation despite domestic time constraints.</t>
+  </si>
+  <si>
+    <t>Subject-specific training workshops are more impactful than general pedagogical sessions.</t>
+  </si>
+  <si>
+    <t>Teacher recommends short WhatsApp summary infographics post-training workshops.</t>
+  </si>
+  <si>
+    <t>Observation feedback delivered privately builds teacher confidence and openness to improvement.</t>
+  </si>
+  <si>
+    <t>Teacher highlights the role of structured accountability in driving continuous professional growth.</t>
+  </si>
+  <si>
+    <t>Integrated offline and online training approach supports ongoing teacher skill development.</t>
   </si>
   <si>
     <t>Implement support staff to alleviate administrative burdens on the headmaster.</t>
@@ -869,141 +869,6 @@
   </si>
   <si>
     <t>Reduce the number of non-teaching duties assigned to actively participating teachers.</t>
-  </si>
-  <si>
-    <t>Name of the interviewer: Rashmi Mishra | Name of the note-taker: Vaibhav Tambe | Date of the interview: 2026-06-10 0:00:00 | Subject taught by teacher: Social Science | Key observation note on teacher's daily engagement: Teacher is also headmaster therefore he highly engaged in academic and non-acad</t>
-  </si>
-  <si>
-    <t>Name of the interviewer: Ritesh Pandey | Name of the note-taker: Vaibhav Kurwade | Date of the interview: 2026-06-10 0:00:00 | Subject taught by teacher: Social Science | Key observation note on teacher's daily engagement: Initially teacher got confused with term activity, so he started explaining t</t>
-  </si>
-  <si>
-    <t>Name of the interviewer: Rajesh Solanki | Name of the note-taker: Shalu Sharma | Date of the interview: 2026-06-11 0:00:00 | Subject taught by teacher: Hindi Social Science | Key observation note on teacher's daily engagement: The teacher said that she is taking all 6 classes everyday but she also i</t>
-  </si>
-  <si>
-    <t>Name of the interviewer: Pushpendra Singh | Date of the interview: 2026-06-10 0:00:00 | Subject taught by teacher: Social Science | Key observation note on teacher's daily engagement: Engaged in academic duties such as teaching also engaged in non-academic work.</t>
-  </si>
-  <si>
-    <t>Name of the interviewer: Dharmendra Mishra | Name of the note-taker: Bhanu Priya | Date of the interview: 2026-06-10 0:00:00 | Subject taught by teacher: Maths Science | Key observation note on teacher's daily engagement: Key observation note on daily engagment 1. Curios and hardworking teacher 2. b</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Name of the interviewer: Shalu Sharma | Name of the note-taker: Rajesh Solanki | Date of the interview: 2026-06-12 0:00:00 | Subject taught by teacher: Maths Science | Key observation note on teacher's daily engagement: the teacher started the conversation with the word Purvgyaan indicating that he </t>
-  </si>
-  <si>
-    <t>Name of the interviewer: Rashmi Mishra | Name of the note-taker: Vaibhav Tambe | Date of the interview: 2026-06-12 0:00:00 | Key observation note on teacher's daily engagement: teacher every 3 day visit door to door for student follow-up. also most of time she been involved to fill various studen</t>
-  </si>
-  <si>
-    <t>Name of the interviewer: Ritesh Pandey | Name of the note-taker: Vaibhav Kurwade | Date of the interview: 2026-06-11 0:00:00 | Subject taught by teacher: Hindi Social Science Sanskrit | Key observation note on teacher's daily engagement: Overall teacher do both types of works, also if we look at the</t>
-  </si>
-  <si>
-    <t>Name of the interviewer: Ritesh Pandey | Name of the note-taker: Vaibhav Kurwade | Date of the interview: 2026-06-12 0:00:00 | Subject taught by teacher: Social Science | Key observation note on teacher's daily engagement: Teacher mainly do a academic activity but based on the need teacher need to c</t>
-  </si>
-  <si>
-    <t>Name of the interviewer: Rahul Kumar | Name of the note-taker: Ashish Nigam | Date of the interview: 2026-06-11 0:00:00 | Key observation note on teacher's daily engagement: largely 50% academic and 50% non-academic works.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Name of the interviewer: Rahul Kumar | Name of the note-taker: Ashish Nigam | Date of the interview: 2026-06-12 0:00:00 | Key observation note on teacher's daily engagement: Teachers generally teach four classes each day, and the remaining time is often spent on non-academic responsibilities. </t>
-  </si>
-  <si>
-    <t>Name of the interviewer: Rashmi Mishra | Name of the note-taker: Rajshree Behera | Date of the interview: 2026-06-11 0:00:00 | Subject taught by teacher: Social Science Sanskrit | Key observation note on teacher's daily engagement: Teacher looked very proud in stating that he tries to dedicate certa</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Name of the interviewer: Naushad Mirza | Name of the note-taker: Deeksha Singh | Date of the interview: 2026-06-10 0:00:00 | Key observation note on teacher's daily engagement: During the conversation, it appeared that he was mindful of presenting his school and team positively. He frequently hig | </t>
-  </si>
-  <si>
-    <t>Name of the interviewer: Pushpendra Singh | Date of the interview: 2026-06-15 0:00:00 | Subject taught by teacher: Hindi Social Science | Key observation note on teacher's daily engagement: The teacher is involved in both teaching and schoolwork. Along with taking classes, the teacher also handles a</t>
-  </si>
-  <si>
-    <t>Name of the interviewer: Rahul Kumar | Name of the note-taker: Ashish Nigam | Date of the interview: 2026-06-15 0:00:00 | Subject taught by teacher: Social Science | Key observation note on teacher's daily engagement: Apart from teaching six classes daily and checking copies, he is also engaged in n</t>
-  </si>
-  <si>
-    <t>Name of the interviewer: Ritesh Pandey | Name of the note-taker: Naushad Mirza | District of respondent teacher: Chhindwara | Date of the interview: 2026-06-16 0:00:00 | Subject taught by teacher: Maths Science | Key observation note on teacher's daily engagement: He is not engagining in other activ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Name of the interviewer: Rashmi Mishra | Name of the note-taker: Vaibhav Tambe | Date of the interview: 2026-06-15 0:00:00 | Subject taught by teacher: Social Science | Key observation note on teacher's daily engagement: white sharing teacher showed the concern about having a only teacher at school </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Name of the interviewer: Rashmi Mishra | Name of the note-taker: Vaibhav Tambe | Date of the interview: 2026-06-16 0:00:00 | Key observation note on teacher's daily engagement: As the Headmaster and sole teacher in the school, the respondent manages both academic and administrative responsibiliti | </t>
-  </si>
-  <si>
-    <t>Name of the interviewer: Vaibhav Kurwade | District of respondent teacher: Narsinghpur | Date of the interview: 2026-06-15 0:00:00 | Subject taught by teacher: Social Science Sanskrit | Key observation note on teacher's daily engagement: Strong focus on holistic student development. Effective integr</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Name of the interviewer: Rahul Kumar | Name of the note-taker: Devendra Sharma | Date of the interview: 2026-06-09 0:00:00 | Subject taught by teacher: Social Science | Key observation note on teacher's daily engagement: it looks like that she worked as a typical teacher of government school. | Key </t>
-  </si>
-  <si>
-    <t>Name of the interviewer: Vaibhav Kurwade | Date of the interview: 2026-06-16 0:00:00 | Subject taught by teacher: English Social Science | Key observation note on teacher's daily engagement: Non-academic responsibilities are not fixed and depend on school requirements. These responsibilities often a</t>
-  </si>
-  <si>
-    <t>Name of the interviewer: Pushpendra Singh | Date of the interview: 2026-06-16 0:00:00 | Subject taught by teacher: Maths Science | Key observation note on teacher's daily engagement: The teacher spends most of the day engaged in classroom teaching and student learning activities. Regular attendance,</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Name of the interviewer: Rashmi Mishra | Name of the note-taker: Vaibhav Tambe | Date of the interview: 2026-06-17 0:00:00 | Subject taught by teacher: Hindi Social Science | Key observation note on teacher's daily engagement: Limited staffing has increased the teacher's workload and expanded their </t>
-  </si>
-  <si>
-    <t>Name of the interviewer: Ritesh Pandey | District of respondent teacher: Chhindwara | Date of the interview: 2026-06-18 0:00:00 | Key observation note on teacher's daily engagement: She was taking 6 classes in a day. She had adtional duties to attend providing data to officials, she was doing online</t>
-  </si>
-  <si>
-    <t>Name of the interviewer: Ritesh Pandey | District of respondent teacher: Chhindwara | Date of the interview: 2026-06-19 0:00:00 | Key observation note on teacher's daily engagement: He says that he is taking classes, doing administrative work, and manitaining relationship with the community. | Key o</t>
-  </si>
-  <si>
-    <t>Name of the interviewer: Ritesh Pandey | Date of the interview: 2026-06-20 0:00:00 | Subject taught by teacher: Maths Science | Key observation note on teacher's daily engagement: she was concerned about completing course of children. | Key observation notes Annual Engagement: She was confused for t</t>
-  </si>
-  <si>
-    <t>Name of the interviewer: Pushpendra Singh | Date of the interview: 2026-06-19 0:00:00 | Subject taught by teacher: Hindi English | Key observation note on teacher's daily engagement: The teacher spends most of the day teaching students. However, the teacher also has to do many office and record-rela</t>
-  </si>
-  <si>
-    <t>Name of the interviewer: Rahul Kumar | Name of the note-taker: Ashish Nigam | Date of the interview: 2026-06-16 0:00:00 | Subject taught by teacher: Social Science Sanskrit | Key observation note on teacher's daily engagement: 60 percent of the time has been spent on academic work. | Key observation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Name of the interviewer: Rahul Kumar | Name of the note-taker: Sonali Patidar | Date of the interview: 2026-06-19 0:00:00 | Key observation note on teacher's daily engagement: according to response of teachers its look like a duty of typical govt teachers. | Key observation notes Annual Engagement: </t>
-  </si>
-  <si>
-    <t>Name of the interviewer: Aishwarya Yadav | Date of the interview: 2026-06-15 0:00:00 | Subject taught by teacher: Maths Science | Key observation note on teacher's daily engagement: The teacher spends some time on non academic tasks like completing the MDM register daily but when it comes to complet</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Name of the interviewer: Aishwarya Yadav | Name of the note-taker: Bhanu Priya | Date of the interview: 2026-06-22 0:00:00 | Subject taught by teacher: Maths Science | Key observation note on teacher's daily engagement: 6 period of classes each day, the teacher felt pressure about the official task </t>
-  </si>
-  <si>
-    <t>Name of the interviewer: Naushad Mirza | Name of the note-taker: Deeksha Singh | Date of the interview: 2026-06-09 0:00:00 | Subject taught by teacher: Social Science | Key observation note on teacher's daily engagement: This teacher teaches Social Science (SST) to Grades 9 and 10. Although he is of</t>
-  </si>
-  <si>
-    <t>Name of the interviewer: Naushad Mirza | Name of the note-taker: Bhanu Priya | Date of the interview: 2026-06-18 0:00:00 | Key observation note on teacher's daily engagement: The teacher plays a role of HM and  ensures that the classes are schedule on time and no classes are free, all the class | Ke</t>
-  </si>
-  <si>
-    <t>Name of the interviewer: Rajshree Behera | Name of the note-taker: Jay Prakash | Date of the interview: 2026-06-19 0:00:00 | Subject taught by teacher: Maths Science | Key observation note on teacher's daily engagement: The teacher was looking a bit nervous in the beginning, and was hesitating a lit</t>
-  </si>
-  <si>
-    <t>Name of the interviewer: Aishwarya Yadav | Date of the interview: 2026-06-19 0:00:00 | Subject taught by teacher: Social Science | Key observation note on teacher's daily engagement: The teacher was not able to share a clear picture of what an average day looks like. The teacher shared that he had t</t>
-  </si>
-  <si>
-    <t>Name of the interviewer: Rajshree Behera | District of respondent teacher: Ashoknagar | Date of the interview: 2026-06-18 0:00:00 | Subject taught by teacher: Social Science | Key observation note on teacher's daily engagement: The teacher is happy, motivated, and emotionally connected with children</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Name of the interviewer: Ritesh Pandey | Name of the note-taker: Vaibhav Kurwade | Date of the interview: 2026-06-13 0:00:00 | Key observation note on teacher's daily engagement: Teacher mainly engaged in academic activities. | Key observation notes Annual Engagement: Teacher took part in in person </t>
-  </si>
-  <si>
-    <t>Name of the interviewer: Naushad Mirza | Name of the note-taker: Pushpendra Singh | Date of the interview: 2026-06-12 0:00:00 | Subject taught by teacher: Social Science Sanskrit | Key observation note on teacher's daily engagement: The teacher dedicated most of his time to classroom teaching and ma</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Name of the note-taker: Vaibhav Kurwade | Date of the interview: 2026-06-18 0:00:00 | Subject taught by teacher: Hindi Maths | Key observation note on teacher's daily engagement: Teacher appeared actively engaged in routine classroom teaching and school activities. She balances instructional respon </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Name of the note-taker: Vaibhav Kurwade | Date of the interview: 2026-06-19 0:00:00 | Subject taught by teacher: English Sanskrit Science | Key observation note on teacher's daily engagement: Teacher need to do both types of work but  the data related work she mainly complete at the home, there was </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Name of the interviewer: Aishwarya Yadav | Name of the note-taker: Shalu Sharma | Date of the interview: 2026-06-16 0:00:00 | Subject taught by teacher: Hindi English | Key observation note on teacher's daily engagement: He knew a lot of terms used in CLSS | Key observation notes Annual Engagement: </t>
-  </si>
-  <si>
-    <t>Name of the interviewer: Aishwarya Yadav | Name of the note-taker: Vaibhav Tambe | District of respondent teacher: Narmadapuram | Date of the interview: 2026-06-24 0:00:00 | Key observation note on teacher's daily engagement: Teacher repeatedly referred to his multiple responsibilities as Headmaster</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Name of the interviewer: Dharmendra Mishra | Name of the note-taker: Deeksha Singh | Date of the interview: 2026-06-11 0:00:00 | Subject taught by teacher: Social Science Other | Key observation note on teacher's daily engagement: He was a teacher nearnin retirement, and he had many questions about </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Name of the interviewer: Bidisha Bose | Date of the interview: 2026-06-18 0:00:00 | Subject taught by teacher: Maths Science | Key observation note on teacher's daily engagement: It seemed like there was no regular schedule at school. It was dependent majorly on the availability of the teacher and  </t>
-  </si>
-  <si>
-    <t>Name of the interviewer: Shalu Sharma | Name of the note-taker: Bidisha Bose | Date of the interview: 2026-06-15 0:00:00 | Subject taught by teacher: Hindi English Maths Science | Key observation note on teacher's daily engagement: he is a promoted middle school teacher but working as a primary teac</t>
   </si>
 </sst>
 </file>
@@ -1387,7 +1252,7 @@
         <v>226</v>
       </c>
       <c r="H2" t="s">
-        <v>285</v>
+        <v>166</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -1413,7 +1278,7 @@
         <v>227</v>
       </c>
       <c r="H3" t="s">
-        <v>286</v>
+        <v>167</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -1465,7 +1330,7 @@
         <v>229</v>
       </c>
       <c r="H5" t="s">
-        <v>287</v>
+        <v>169</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -1491,7 +1356,7 @@
         <v>230</v>
       </c>
       <c r="H6" t="s">
-        <v>288</v>
+        <v>170</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -1517,7 +1382,7 @@
         <v>231</v>
       </c>
       <c r="H7" t="s">
-        <v>289</v>
+        <v>171</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -1543,7 +1408,7 @@
         <v>232</v>
       </c>
       <c r="H8" t="s">
-        <v>290</v>
+        <v>172</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -1569,7 +1434,7 @@
         <v>233</v>
       </c>
       <c r="H9" t="s">
-        <v>291</v>
+        <v>173</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -1595,7 +1460,7 @@
         <v>234</v>
       </c>
       <c r="H10" t="s">
-        <v>292</v>
+        <v>174</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -1647,7 +1512,7 @@
         <v>236</v>
       </c>
       <c r="H12" t="s">
-        <v>293</v>
+        <v>176</v>
       </c>
     </row>
     <row r="13" spans="1:8">
@@ -1699,7 +1564,7 @@
         <v>237</v>
       </c>
       <c r="H14" t="s">
-        <v>294</v>
+        <v>178</v>
       </c>
     </row>
     <row r="15" spans="1:8">
@@ -1725,7 +1590,7 @@
         <v>238</v>
       </c>
       <c r="H15" t="s">
-        <v>295</v>
+        <v>179</v>
       </c>
     </row>
     <row r="16" spans="1:8">
@@ -1751,7 +1616,7 @@
         <v>239</v>
       </c>
       <c r="H16" t="s">
-        <v>296</v>
+        <v>180</v>
       </c>
     </row>
     <row r="17" spans="1:8">
@@ -1777,7 +1642,7 @@
         <v>240</v>
       </c>
       <c r="H17" t="s">
-        <v>297</v>
+        <v>181</v>
       </c>
     </row>
     <row r="18" spans="1:8">
@@ -1803,7 +1668,7 @@
         <v>241</v>
       </c>
       <c r="H18" t="s">
-        <v>298</v>
+        <v>182</v>
       </c>
     </row>
     <row r="19" spans="1:8">
@@ -1855,7 +1720,7 @@
         <v>243</v>
       </c>
       <c r="H20" t="s">
-        <v>299</v>
+        <v>184</v>
       </c>
     </row>
     <row r="21" spans="1:8">
@@ -1907,7 +1772,7 @@
         <v>245</v>
       </c>
       <c r="H22" t="s">
-        <v>300</v>
+        <v>186</v>
       </c>
     </row>
     <row r="23" spans="1:8">
@@ -1933,7 +1798,7 @@
         <v>246</v>
       </c>
       <c r="H23" t="s">
-        <v>301</v>
+        <v>187</v>
       </c>
     </row>
     <row r="24" spans="1:8">
@@ -1959,7 +1824,7 @@
         <v>247</v>
       </c>
       <c r="H24" t="s">
-        <v>302</v>
+        <v>188</v>
       </c>
     </row>
     <row r="25" spans="1:8">
@@ -1985,7 +1850,7 @@
         <v>248</v>
       </c>
       <c r="H25" t="s">
-        <v>303</v>
+        <v>189</v>
       </c>
     </row>
     <row r="26" spans="1:8">
@@ -2011,7 +1876,7 @@
         <v>249</v>
       </c>
       <c r="H26" t="s">
-        <v>304</v>
+        <v>190</v>
       </c>
     </row>
     <row r="27" spans="1:8">
@@ -2063,7 +1928,7 @@
         <v>251</v>
       </c>
       <c r="H28" t="s">
-        <v>305</v>
+        <v>192</v>
       </c>
     </row>
     <row r="29" spans="1:8">
@@ -2089,7 +1954,7 @@
         <v>252</v>
       </c>
       <c r="H29" t="s">
-        <v>306</v>
+        <v>193</v>
       </c>
     </row>
     <row r="30" spans="1:8">
@@ -2115,7 +1980,7 @@
         <v>253</v>
       </c>
       <c r="H30" t="s">
-        <v>307</v>
+        <v>194</v>
       </c>
     </row>
     <row r="31" spans="1:8">
@@ -2141,7 +2006,7 @@
         <v>254</v>
       </c>
       <c r="H31" t="s">
-        <v>308</v>
+        <v>195</v>
       </c>
     </row>
     <row r="32" spans="1:8">
@@ -2297,7 +2162,7 @@
         <v>260</v>
       </c>
       <c r="H37" t="s">
-        <v>309</v>
+        <v>201</v>
       </c>
     </row>
     <row r="38" spans="1:8">
@@ -2375,7 +2240,7 @@
         <v>263</v>
       </c>
       <c r="H40" t="s">
-        <v>310</v>
+        <v>204</v>
       </c>
     </row>
     <row r="41" spans="1:8">
@@ -2427,7 +2292,7 @@
         <v>265</v>
       </c>
       <c r="H42" t="s">
-        <v>311</v>
+        <v>206</v>
       </c>
     </row>
     <row r="43" spans="1:8">
@@ -2453,7 +2318,7 @@
         <v>266</v>
       </c>
       <c r="H43" t="s">
-        <v>312</v>
+        <v>207</v>
       </c>
     </row>
     <row r="44" spans="1:8">
@@ -2479,7 +2344,7 @@
         <v>267</v>
       </c>
       <c r="H44" t="s">
-        <v>313</v>
+        <v>208</v>
       </c>
     </row>
     <row r="45" spans="1:8">
@@ -2505,7 +2370,7 @@
         <v>268</v>
       </c>
       <c r="H45" t="s">
-        <v>314</v>
+        <v>209</v>
       </c>
     </row>
     <row r="46" spans="1:8">
@@ -2531,7 +2396,7 @@
         <v>269</v>
       </c>
       <c r="H46" t="s">
-        <v>315</v>
+        <v>210</v>
       </c>
     </row>
     <row r="47" spans="1:8">
@@ -2557,7 +2422,7 @@
         <v>270</v>
       </c>
       <c r="H47" t="s">
-        <v>316</v>
+        <v>211</v>
       </c>
     </row>
     <row r="48" spans="1:8">
@@ -2583,7 +2448,7 @@
         <v>271</v>
       </c>
       <c r="H48" t="s">
-        <v>317</v>
+        <v>212</v>
       </c>
     </row>
     <row r="49" spans="1:8">
@@ -2609,7 +2474,7 @@
         <v>272</v>
       </c>
       <c r="H49" t="s">
-        <v>318</v>
+        <v>213</v>
       </c>
     </row>
     <row r="50" spans="1:8">
@@ -2635,7 +2500,7 @@
         <v>273</v>
       </c>
       <c r="H50" t="s">
-        <v>319</v>
+        <v>214</v>
       </c>
     </row>
     <row r="51" spans="1:8">
@@ -2661,7 +2526,7 @@
         <v>274</v>
       </c>
       <c r="H51" t="s">
-        <v>320</v>
+        <v>215</v>
       </c>
     </row>
     <row r="52" spans="1:8">
@@ -2713,7 +2578,7 @@
         <v>276</v>
       </c>
       <c r="H53" t="s">
-        <v>321</v>
+        <v>217</v>
       </c>
     </row>
     <row r="54" spans="1:8">
@@ -2739,7 +2604,7 @@
         <v>277</v>
       </c>
       <c r="H54" t="s">
-        <v>322</v>
+        <v>218</v>
       </c>
     </row>
     <row r="55" spans="1:8">
@@ -2765,7 +2630,7 @@
         <v>278</v>
       </c>
       <c r="H55" t="s">
-        <v>323</v>
+        <v>219</v>
       </c>
     </row>
     <row r="56" spans="1:8">
@@ -2791,7 +2656,7 @@
         <v>279</v>
       </c>
       <c r="H56" t="s">
-        <v>324</v>
+        <v>220</v>
       </c>
     </row>
     <row r="57" spans="1:8">
@@ -2817,7 +2682,7 @@
         <v>280</v>
       </c>
       <c r="H57" t="s">
-        <v>325</v>
+        <v>221</v>
       </c>
     </row>
     <row r="58" spans="1:8">
@@ -2843,7 +2708,7 @@
         <v>281</v>
       </c>
       <c r="H58" t="s">
-        <v>326</v>
+        <v>222</v>
       </c>
     </row>
     <row r="59" spans="1:8">
@@ -2869,7 +2734,7 @@
         <v>282</v>
       </c>
       <c r="H59" t="s">
-        <v>327</v>
+        <v>223</v>
       </c>
     </row>
     <row r="60" spans="1:8">
@@ -2895,7 +2760,7 @@
         <v>283</v>
       </c>
       <c r="H60" t="s">
-        <v>328</v>
+        <v>224</v>
       </c>
     </row>
     <row r="61" spans="1:8">
@@ -2921,7 +2786,7 @@
         <v>284</v>
       </c>
       <c r="H61" t="s">
-        <v>329</v>
+        <v>225</v>
       </c>
     </row>
   </sheetData>

</xml_diff>